<commit_message>
results flex ops with updated opex var mea
</commit_message>
<xml_diff>
--- a/dataCaseStudy_Cement/raw_results/flexible_ops/Summary.xlsx
+++ b/dataCaseStudy_Cement/raw_results/flexible_ops/Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE231"/>
+  <dimension ref="A1:AE243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24272,6 +24272,1242 @@
       <c r="AE231" t="inlineStr">
         <is>
           <t>dataCaseStudy_Cement\raw_results\flexible_ops\20260331162810_mea_inflex_std_2_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>198380143.7954721</v>
+      </c>
+      <c r="B232" t="n">
+        <v>15822294.2146771</v>
+      </c>
+      <c r="C232" t="n">
+        <v>5950072.294242878</v>
+      </c>
+      <c r="D232" t="n">
+        <v>9948608.915923037</v>
+      </c>
+      <c r="E232" t="n">
+        <v>0</v>
+      </c>
+      <c r="F232" t="n">
+        <v>25770903.13060014</v>
+      </c>
+      <c r="G232" t="n">
+        <v>5950072.294242878</v>
+      </c>
+      <c r="H232" t="n">
+        <v>157546783.7957529</v>
+      </c>
+      <c r="I232" t="n">
+        <v>0</v>
+      </c>
+      <c r="J232" t="n">
+        <v>0</v>
+      </c>
+      <c r="K232" t="n">
+        <v>0</v>
+      </c>
+      <c r="L232" t="n">
+        <v>9112384.574876238</v>
+      </c>
+      <c r="M232" t="n">
+        <v>198380143.7954721</v>
+      </c>
+      <c r="N232" t="n">
+        <v>60756.06478760556</v>
+      </c>
+      <c r="O232" t="n">
+        <v>0</v>
+      </c>
+      <c r="P232" t="n">
+        <v>60756.06478760556</v>
+      </c>
+      <c r="Q232" t="n">
+        <v>60749.23049917545</v>
+      </c>
+      <c r="R232" t="n">
+        <v>0</v>
+      </c>
+      <c r="S232" t="n">
+        <v>0</v>
+      </c>
+      <c r="T232" t="n">
+        <v>0</v>
+      </c>
+      <c r="U232" t="n">
+        <v>6.834288431157251</v>
+      </c>
+      <c r="V232" t="n">
+        <v>10462.08700013161</v>
+      </c>
+      <c r="W232" t="n">
+        <v>193542247.1490416</v>
+      </c>
+      <c r="X232" t="n">
+        <v>198380143.7954721</v>
+      </c>
+      <c r="Y232" t="n">
+        <v>4837896.646430582</v>
+      </c>
+      <c r="Z232" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA232" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB232" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC232" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD232" t="inlineStr">
+        <is>
+          <t>mea_std_1_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE232" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\flexible_ops\20260424213421_mea_std_1_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>216929866.9238391</v>
+      </c>
+      <c r="B233" t="n">
+        <v>15828554.68961275</v>
+      </c>
+      <c r="C233" t="n">
+        <v>5951746.544758596</v>
+      </c>
+      <c r="D233" t="n">
+        <v>9943373.656616133</v>
+      </c>
+      <c r="E233" t="n">
+        <v>0</v>
+      </c>
+      <c r="F233" t="n">
+        <v>25771928.34622888</v>
+      </c>
+      <c r="G233" t="n">
+        <v>5951746.544758596</v>
+      </c>
+      <c r="H233" t="n">
+        <v>175939023.922078</v>
+      </c>
+      <c r="I233" t="n">
+        <v>0</v>
+      </c>
+      <c r="J233" t="n">
+        <v>0</v>
+      </c>
+      <c r="K233" t="n">
+        <v>0</v>
+      </c>
+      <c r="L233" t="n">
+        <v>9267168.110773632</v>
+      </c>
+      <c r="M233" t="n">
+        <v>216929866.9238391</v>
+      </c>
+      <c r="N233" t="n">
+        <v>61787.94212829431</v>
+      </c>
+      <c r="O233" t="n">
+        <v>0</v>
+      </c>
+      <c r="P233" t="n">
+        <v>61787.94212829431</v>
+      </c>
+      <c r="Q233" t="n">
+        <v>61781.12073849125</v>
+      </c>
+      <c r="R233" t="n">
+        <v>0</v>
+      </c>
+      <c r="S233" t="n">
+        <v>0</v>
+      </c>
+      <c r="T233" t="n">
+        <v>0</v>
+      </c>
+      <c r="U233" t="n">
+        <v>6.821389803165927</v>
+      </c>
+      <c r="V233" t="n">
+        <v>1342.444999933243</v>
+      </c>
+      <c r="W233" t="n">
+        <v>212187783.2033313</v>
+      </c>
+      <c r="X233" t="n">
+        <v>216929866.9238391</v>
+      </c>
+      <c r="Y233" t="n">
+        <v>4742083.720507801</v>
+      </c>
+      <c r="Z233" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA233" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB233" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC233" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD233" t="inlineStr">
+        <is>
+          <t>mea_std_1_el_price_107</t>
+        </is>
+      </c>
+      <c r="AE233" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\flexible_ops\20260425003144_mea_std_1_el_price_107</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>232401125.9793854</v>
+      </c>
+      <c r="B234" t="n">
+        <v>0</v>
+      </c>
+      <c r="C234" t="n">
+        <v>0</v>
+      </c>
+      <c r="D234" t="n">
+        <v>0</v>
+      </c>
+      <c r="E234" t="n">
+        <v>0</v>
+      </c>
+      <c r="F234" t="n">
+        <v>0</v>
+      </c>
+      <c r="G234" t="n">
+        <v>0</v>
+      </c>
+      <c r="H234" t="n">
+        <v>141277280.2306274</v>
+      </c>
+      <c r="I234" t="n">
+        <v>0</v>
+      </c>
+      <c r="J234" t="n">
+        <v>0</v>
+      </c>
+      <c r="K234" t="n">
+        <v>0</v>
+      </c>
+      <c r="L234" t="n">
+        <v>91123845.74875793</v>
+      </c>
+      <c r="M234" t="n">
+        <v>232401125.9793854</v>
+      </c>
+      <c r="N234" t="n">
+        <v>607492.3049917968</v>
+      </c>
+      <c r="O234" t="n">
+        <v>0</v>
+      </c>
+      <c r="P234" t="n">
+        <v>607492.3049917968</v>
+      </c>
+      <c r="Q234" t="n">
+        <v>607492.3049917665</v>
+      </c>
+      <c r="R234" t="n">
+        <v>0</v>
+      </c>
+      <c r="S234" t="n">
+        <v>0</v>
+      </c>
+      <c r="T234" t="n">
+        <v>0</v>
+      </c>
+      <c r="U234" t="n">
+        <v>0</v>
+      </c>
+      <c r="V234" t="n">
+        <v>2153.633999824524</v>
+      </c>
+      <c r="W234" t="n">
+        <v>226084153.7089693</v>
+      </c>
+      <c r="X234" t="n">
+        <v>232401125.9793854</v>
+      </c>
+      <c r="Y234" t="n">
+        <v>6316972.270416081</v>
+      </c>
+      <c r="Z234" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA234" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB234" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC234" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD234" t="inlineStr">
+        <is>
+          <t>mea_std_1_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE234" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\flexible_ops\20260425005652_mea_std_1_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>198225520.6663301</v>
+      </c>
+      <c r="B235" t="n">
+        <v>15828554.68961276</v>
+      </c>
+      <c r="C235" t="n">
+        <v>5951746.544758598</v>
+      </c>
+      <c r="D235" t="n">
+        <v>9950906.361202728</v>
+      </c>
+      <c r="E235" t="n">
+        <v>0</v>
+      </c>
+      <c r="F235" t="n">
+        <v>25779461.05081549</v>
+      </c>
+      <c r="G235" t="n">
+        <v>5951746.544758598</v>
+      </c>
+      <c r="H235" t="n">
+        <v>157381928.4958803</v>
+      </c>
+      <c r="I235" t="n">
+        <v>0</v>
+      </c>
+      <c r="J235" t="n">
+        <v>0</v>
+      </c>
+      <c r="K235" t="n">
+        <v>0</v>
+      </c>
+      <c r="L235" t="n">
+        <v>9112384.574875711</v>
+      </c>
+      <c r="M235" t="n">
+        <v>198225520.6663301</v>
+      </c>
+      <c r="N235" t="n">
+        <v>60756.06478762635</v>
+      </c>
+      <c r="O235" t="n">
+        <v>0</v>
+      </c>
+      <c r="P235" t="n">
+        <v>60756.06478762635</v>
+      </c>
+      <c r="Q235" t="n">
+        <v>60749.23049917664</v>
+      </c>
+      <c r="R235" t="n">
+        <v>0</v>
+      </c>
+      <c r="S235" t="n">
+        <v>0</v>
+      </c>
+      <c r="T235" t="n">
+        <v>0</v>
+      </c>
+      <c r="U235" t="n">
+        <v>6.834288431157373</v>
+      </c>
+      <c r="V235" t="n">
+        <v>914.0090000629425</v>
+      </c>
+      <c r="W235" t="n">
+        <v>193458936.7299272</v>
+      </c>
+      <c r="X235" t="n">
+        <v>198225520.6663301</v>
+      </c>
+      <c r="Y235" t="n">
+        <v>4766583.936402828</v>
+      </c>
+      <c r="Z235" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA235" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB235" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC235" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD235" t="inlineStr">
+        <is>
+          <t>mea_std_2_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE235" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\flexible_ops\20260425013547_mea_std_2_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>215851260.926798</v>
+      </c>
+      <c r="B236" t="n">
+        <v>15822294.21472696</v>
+      </c>
+      <c r="C236" t="n">
+        <v>5950072.294242923</v>
+      </c>
+      <c r="D236" t="n">
+        <v>9904011.551154803</v>
+      </c>
+      <c r="E236" t="n">
+        <v>0</v>
+      </c>
+      <c r="F236" t="n">
+        <v>25726305.76588176</v>
+      </c>
+      <c r="G236" t="n">
+        <v>5950072.294242923</v>
+      </c>
+      <c r="H236" t="n">
+        <v>174146102.6292823</v>
+      </c>
+      <c r="I236" t="n">
+        <v>0</v>
+      </c>
+      <c r="J236" t="n">
+        <v>0</v>
+      </c>
+      <c r="K236" t="n">
+        <v>0</v>
+      </c>
+      <c r="L236" t="n">
+        <v>10028780.23739106</v>
+      </c>
+      <c r="M236" t="n">
+        <v>215851260.926798</v>
+      </c>
+      <c r="N236" t="n">
+        <v>66865.29283806655</v>
+      </c>
+      <c r="O236" t="n">
+        <v>0</v>
+      </c>
+      <c r="P236" t="n">
+        <v>66865.29283806655</v>
+      </c>
+      <c r="Q236" t="n">
+        <v>66858.53491594146</v>
+      </c>
+      <c r="R236" t="n">
+        <v>0</v>
+      </c>
+      <c r="S236" t="n">
+        <v>0</v>
+      </c>
+      <c r="T236" t="n">
+        <v>0</v>
+      </c>
+      <c r="U236" t="n">
+        <v>6.757922125947767</v>
+      </c>
+      <c r="V236" t="n">
+        <v>1621.40499997139</v>
+      </c>
+      <c r="W236" t="n">
+        <v>211429752.3127332</v>
+      </c>
+      <c r="X236" t="n">
+        <v>215851260.926798</v>
+      </c>
+      <c r="Y236" t="n">
+        <v>4421508.614064842</v>
+      </c>
+      <c r="Z236" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA236" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB236" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC236" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD236" t="inlineStr">
+        <is>
+          <t>mea_std_2_el_price_107</t>
+        </is>
+      </c>
+      <c r="AE236" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\flexible_ops\20260425015348_mea_std_2_el_price_107</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>226659646.0685059</v>
+      </c>
+      <c r="B237" t="n">
+        <v>15834820.84864306</v>
+      </c>
+      <c r="C237" t="n">
+        <v>5953422.254316006</v>
+      </c>
+      <c r="D237" t="n">
+        <v>9599594.119778559</v>
+      </c>
+      <c r="E237" t="n">
+        <v>0</v>
+      </c>
+      <c r="F237" t="n">
+        <v>25434414.96842162</v>
+      </c>
+      <c r="G237" t="n">
+        <v>5953422.254316006</v>
+      </c>
+      <c r="H237" t="n">
+        <v>178893339.8386377</v>
+      </c>
+      <c r="I237" t="n">
+        <v>0</v>
+      </c>
+      <c r="J237" t="n">
+        <v>0</v>
+      </c>
+      <c r="K237" t="n">
+        <v>0</v>
+      </c>
+      <c r="L237" t="n">
+        <v>16378469.00713065</v>
+      </c>
+      <c r="M237" t="n">
+        <v>226659646.0685059</v>
+      </c>
+      <c r="N237" t="n">
+        <v>109196.0221622654</v>
+      </c>
+      <c r="O237" t="n">
+        <v>0</v>
+      </c>
+      <c r="P237" t="n">
+        <v>109196.0221622654</v>
+      </c>
+      <c r="Q237" t="n">
+        <v>109189.7933808706</v>
+      </c>
+      <c r="R237" t="n">
+        <v>0</v>
+      </c>
+      <c r="S237" t="n">
+        <v>0</v>
+      </c>
+      <c r="T237" t="n">
+        <v>0</v>
+      </c>
+      <c r="U237" t="n">
+        <v>6.228781395136024</v>
+      </c>
+      <c r="V237" t="n">
+        <v>7548.073000192642</v>
+      </c>
+      <c r="W237" t="n">
+        <v>223495083.2110209</v>
+      </c>
+      <c r="X237" t="n">
+        <v>226659646.0685059</v>
+      </c>
+      <c r="Y237" t="n">
+        <v>3164562.857484996</v>
+      </c>
+      <c r="Z237" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA237" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB237" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC237" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD237" t="inlineStr">
+        <is>
+          <t>mea_std_2_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE237" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\flexible_ops\20260425022343_mea_std_2_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>198392979.5859249</v>
+      </c>
+      <c r="B238" t="n">
+        <v>15828554.68961275</v>
+      </c>
+      <c r="C238" t="n">
+        <v>5951746.544758594</v>
+      </c>
+      <c r="D238" t="n">
+        <v>9950906.361203149</v>
+      </c>
+      <c r="E238" t="n">
+        <v>0</v>
+      </c>
+      <c r="F238" t="n">
+        <v>25779461.0508159</v>
+      </c>
+      <c r="G238" t="n">
+        <v>5951746.544758594</v>
+      </c>
+      <c r="H238" t="n">
+        <v>157549387.415474</v>
+      </c>
+      <c r="I238" t="n">
+        <v>0</v>
+      </c>
+      <c r="J238" t="n">
+        <v>0</v>
+      </c>
+      <c r="K238" t="n">
+        <v>0</v>
+      </c>
+      <c r="L238" t="n">
+        <v>9112384.574876411</v>
+      </c>
+      <c r="M238" t="n">
+        <v>198392979.5859249</v>
+      </c>
+      <c r="N238" t="n">
+        <v>60756.06478760711</v>
+      </c>
+      <c r="O238" t="n">
+        <v>0</v>
+      </c>
+      <c r="P238" t="n">
+        <v>60756.06478760711</v>
+      </c>
+      <c r="Q238" t="n">
+        <v>60749.23049917634</v>
+      </c>
+      <c r="R238" t="n">
+        <v>0</v>
+      </c>
+      <c r="S238" t="n">
+        <v>0</v>
+      </c>
+      <c r="T238" t="n">
+        <v>0</v>
+      </c>
+      <c r="U238" t="n">
+        <v>6.834288431157366</v>
+      </c>
+      <c r="V238" t="n">
+        <v>3.625</v>
+      </c>
+      <c r="W238" t="n">
+        <v>194156504.7369564</v>
+      </c>
+      <c r="X238" t="n">
+        <v>198392979.5859249</v>
+      </c>
+      <c r="Y238" t="n">
+        <v>4236474.848968536</v>
+      </c>
+      <c r="Z238" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA238" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB238" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC238" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD238" t="inlineStr">
+        <is>
+          <t>mea_inflex_std_1_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE238" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\flexible_ops\20260425043234_mea_inflex_std_1_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>216929866.9238383</v>
+      </c>
+      <c r="B239" t="n">
+        <v>15828554.68961275</v>
+      </c>
+      <c r="C239" t="n">
+        <v>5951746.544758594</v>
+      </c>
+      <c r="D239" t="n">
+        <v>9943373.656616133</v>
+      </c>
+      <c r="E239" t="n">
+        <v>0</v>
+      </c>
+      <c r="F239" t="n">
+        <v>25771928.34622888</v>
+      </c>
+      <c r="G239" t="n">
+        <v>5951746.544758594</v>
+      </c>
+      <c r="H239" t="n">
+        <v>175939023.9220771</v>
+      </c>
+      <c r="I239" t="n">
+        <v>0</v>
+      </c>
+      <c r="J239" t="n">
+        <v>0</v>
+      </c>
+      <c r="K239" t="n">
+        <v>0</v>
+      </c>
+      <c r="L239" t="n">
+        <v>9267168.110773703</v>
+      </c>
+      <c r="M239" t="n">
+        <v>216929866.9238383</v>
+      </c>
+      <c r="N239" t="n">
+        <v>61787.94212829439</v>
+      </c>
+      <c r="O239" t="n">
+        <v>0</v>
+      </c>
+      <c r="P239" t="n">
+        <v>61787.94212829439</v>
+      </c>
+      <c r="Q239" t="n">
+        <v>61781.12073849163</v>
+      </c>
+      <c r="R239" t="n">
+        <v>0</v>
+      </c>
+      <c r="S239" t="n">
+        <v>0</v>
+      </c>
+      <c r="T239" t="n">
+        <v>0</v>
+      </c>
+      <c r="U239" t="n">
+        <v>6.821389803165925</v>
+      </c>
+      <c r="V239" t="n">
+        <v>3.453999996185303</v>
+      </c>
+      <c r="W239" t="n">
+        <v>212693392.0748695</v>
+      </c>
+      <c r="X239" t="n">
+        <v>216929866.9238383</v>
+      </c>
+      <c r="Y239" t="n">
+        <v>4236474.848968774</v>
+      </c>
+      <c r="Z239" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA239" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB239" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC239" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD239" t="inlineStr">
+        <is>
+          <t>mea_inflex_std_1_el_price_107</t>
+        </is>
+      </c>
+      <c r="AE239" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\flexible_ops\20260425043550_mea_inflex_std_1_el_price_107</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>230740725.8105568</v>
+      </c>
+      <c r="B240" t="n">
+        <v>15828554.68961275</v>
+      </c>
+      <c r="C240" t="n">
+        <v>5951746.544758594</v>
+      </c>
+      <c r="D240" t="n">
+        <v>9872102.682446657</v>
+      </c>
+      <c r="E240" t="n">
+        <v>0</v>
+      </c>
+      <c r="F240" t="n">
+        <v>25700657.3720594</v>
+      </c>
+      <c r="G240" t="n">
+        <v>5951746.544758594</v>
+      </c>
+      <c r="H240" t="n">
+        <v>188356663.4048599</v>
+      </c>
+      <c r="I240" t="n">
+        <v>0</v>
+      </c>
+      <c r="J240" t="n">
+        <v>0</v>
+      </c>
+      <c r="K240" t="n">
+        <v>0</v>
+      </c>
+      <c r="L240" t="n">
+        <v>10731658.48887887</v>
+      </c>
+      <c r="M240" t="n">
+        <v>230740725.8105568</v>
+      </c>
+      <c r="N240" t="n">
+        <v>71551.08927479727</v>
+      </c>
+      <c r="O240" t="n">
+        <v>0</v>
+      </c>
+      <c r="P240" t="n">
+        <v>71551.08927479727</v>
+      </c>
+      <c r="Q240" t="n">
+        <v>71544.3899258593</v>
+      </c>
+      <c r="R240" t="n">
+        <v>0</v>
+      </c>
+      <c r="S240" t="n">
+        <v>0</v>
+      </c>
+      <c r="T240" t="n">
+        <v>0</v>
+      </c>
+      <c r="U240" t="n">
+        <v>6.699348938323829</v>
+      </c>
+      <c r="V240" t="n">
+        <v>3.233000040054321</v>
+      </c>
+      <c r="W240" t="n">
+        <v>226504250.9615883</v>
+      </c>
+      <c r="X240" t="n">
+        <v>230740725.8105568</v>
+      </c>
+      <c r="Y240" t="n">
+        <v>4236474.848968476</v>
+      </c>
+      <c r="Z240" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA240" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB240" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC240" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD240" t="inlineStr">
+        <is>
+          <t>mea_inflex_std_1_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE240" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\flexible_ops\20260425043804_mea_inflex_std_1_el_price_150</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>198225520.6663415</v>
+      </c>
+      <c r="B241" t="n">
+        <v>15828554.68961275</v>
+      </c>
+      <c r="C241" t="n">
+        <v>5951746.544758594</v>
+      </c>
+      <c r="D241" t="n">
+        <v>9950906.361203149</v>
+      </c>
+      <c r="E241" t="n">
+        <v>0</v>
+      </c>
+      <c r="F241" t="n">
+        <v>25779461.0508159</v>
+      </c>
+      <c r="G241" t="n">
+        <v>5951746.544758594</v>
+      </c>
+      <c r="H241" t="n">
+        <v>157381928.4958906</v>
+      </c>
+      <c r="I241" t="n">
+        <v>0</v>
+      </c>
+      <c r="J241" t="n">
+        <v>0</v>
+      </c>
+      <c r="K241" t="n">
+        <v>0</v>
+      </c>
+      <c r="L241" t="n">
+        <v>9112384.574876411</v>
+      </c>
+      <c r="M241" t="n">
+        <v>198225520.6663415</v>
+      </c>
+      <c r="N241" t="n">
+        <v>60756.06478760711</v>
+      </c>
+      <c r="O241" t="n">
+        <v>0</v>
+      </c>
+      <c r="P241" t="n">
+        <v>60756.06478760711</v>
+      </c>
+      <c r="Q241" t="n">
+        <v>60749.23049917634</v>
+      </c>
+      <c r="R241" t="n">
+        <v>0</v>
+      </c>
+      <c r="S241" t="n">
+        <v>0</v>
+      </c>
+      <c r="T241" t="n">
+        <v>0</v>
+      </c>
+      <c r="U241" t="n">
+        <v>6.834288431157366</v>
+      </c>
+      <c r="V241" t="n">
+        <v>4.746999979019165</v>
+      </c>
+      <c r="W241" t="n">
+        <v>193989045.817373</v>
+      </c>
+      <c r="X241" t="n">
+        <v>198225520.6663415</v>
+      </c>
+      <c r="Y241" t="n">
+        <v>4236474.848968416</v>
+      </c>
+      <c r="Z241" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA241" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB241" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC241" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD241" t="inlineStr">
+        <is>
+          <t>mea_inflex_std_2_el_price_50</t>
+        </is>
+      </c>
+      <c r="AE241" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\flexible_ops\20260425044130_mea_inflex_std_2_el_price_50</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>216339245.2149234</v>
+      </c>
+      <c r="B242" t="n">
+        <v>15828554.68961275</v>
+      </c>
+      <c r="C242" t="n">
+        <v>5951746.544758594</v>
+      </c>
+      <c r="D242" t="n">
+        <v>9883112.019919991</v>
+      </c>
+      <c r="E242" t="n">
+        <v>0</v>
+      </c>
+      <c r="F242" t="n">
+        <v>25711666.70953274</v>
+      </c>
+      <c r="G242" t="n">
+        <v>5951746.544758594</v>
+      </c>
+      <c r="H242" t="n">
+        <v>174170395.56268</v>
+      </c>
+      <c r="I242" t="n">
+        <v>0</v>
+      </c>
+      <c r="J242" t="n">
+        <v>0</v>
+      </c>
+      <c r="K242" t="n">
+        <v>0</v>
+      </c>
+      <c r="L242" t="n">
+        <v>10505436.39795206</v>
+      </c>
+      <c r="M242" t="n">
+        <v>216339245.2149234</v>
+      </c>
+      <c r="N242" t="n">
+        <v>70042.96085379274</v>
+      </c>
+      <c r="O242" t="n">
+        <v>0</v>
+      </c>
+      <c r="P242" t="n">
+        <v>70042.96085379274</v>
+      </c>
+      <c r="Q242" t="n">
+        <v>70036.24265301388</v>
+      </c>
+      <c r="R242" t="n">
+        <v>0</v>
+      </c>
+      <c r="S242" t="n">
+        <v>0</v>
+      </c>
+      <c r="T242" t="n">
+        <v>0</v>
+      </c>
+      <c r="U242" t="n">
+        <v>6.718200779234397</v>
+      </c>
+      <c r="V242" t="n">
+        <v>3.592000007629395</v>
+      </c>
+      <c r="W242" t="n">
+        <v>212102770.365955</v>
+      </c>
+      <c r="X242" t="n">
+        <v>216339245.2149234</v>
+      </c>
+      <c r="Y242" t="n">
+        <v>4236474.848968446</v>
+      </c>
+      <c r="Z242" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA242" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB242" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC242" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD242" t="inlineStr">
+        <is>
+          <t>mea_inflex_std_2_el_price_107</t>
+        </is>
+      </c>
+      <c r="AE242" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\flexible_ops\20260425044346_mea_inflex_std_2_el_price_107</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>228409984.2613358</v>
+      </c>
+      <c r="B243" t="n">
+        <v>15828554.68961275</v>
+      </c>
+      <c r="C243" t="n">
+        <v>5951746.544758594</v>
+      </c>
+      <c r="D243" t="n">
+        <v>9496046.891910162</v>
+      </c>
+      <c r="E243" t="n">
+        <v>0</v>
+      </c>
+      <c r="F243" t="n">
+        <v>25324601.58152291</v>
+      </c>
+      <c r="G243" t="n">
+        <v>5951746.544758594</v>
+      </c>
+      <c r="H243" t="n">
+        <v>178674707.2771491</v>
+      </c>
+      <c r="I243" t="n">
+        <v>0</v>
+      </c>
+      <c r="J243" t="n">
+        <v>0</v>
+      </c>
+      <c r="K243" t="n">
+        <v>0</v>
+      </c>
+      <c r="L243" t="n">
+        <v>18458928.85790531</v>
+      </c>
+      <c r="M243" t="n">
+        <v>228409984.2613358</v>
+      </c>
+      <c r="N243" t="n">
+        <v>123065.5811291093</v>
+      </c>
+      <c r="O243" t="n">
+        <v>0</v>
+      </c>
+      <c r="P243" t="n">
+        <v>123065.5811291093</v>
+      </c>
+      <c r="Q243" t="n">
+        <v>123059.5257193684</v>
+      </c>
+      <c r="R243" t="n">
+        <v>0</v>
+      </c>
+      <c r="S243" t="n">
+        <v>0</v>
+      </c>
+      <c r="T243" t="n">
+        <v>0</v>
+      </c>
+      <c r="U243" t="n">
+        <v>6.055409740904965</v>
+      </c>
+      <c r="V243" t="n">
+        <v>3.569999933242798</v>
+      </c>
+      <c r="W243" t="n">
+        <v>224173509.4123673</v>
+      </c>
+      <c r="X243" t="n">
+        <v>228409984.2613358</v>
+      </c>
+      <c r="Y243" t="n">
+        <v>4236474.848968565</v>
+      </c>
+      <c r="Z243" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="AA243" t="inlineStr">
+        <is>
+          <t>costs</t>
+        </is>
+      </c>
+      <c r="AB243" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC243" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD243" t="inlineStr">
+        <is>
+          <t>mea_inflex_std_2_el_price_150</t>
+        </is>
+      </c>
+      <c r="AE243" t="inlineStr">
+        <is>
+          <t>dataCaseStudy_Cement\raw_results\flexible_ops\20260425044731_mea_inflex_std_2_el_price_150</t>
         </is>
       </c>
     </row>

</xml_diff>